<commit_message>
Fix webhook 400 error and pin dependencies
</commit_message>
<xml_diff>
--- a/app version.xlsx
+++ b/app version.xlsx
@@ -4,18 +4,18 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="app.py" sheetId="1" r:id="rId1"/>
-    <sheet name="pinescript" sheetId="2" r:id="rId2"/>
+    <sheet name="MA" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>Version</t>
   </si>
@@ -29,21 +29,12 @@
     <t>Working(Y/N)</t>
   </si>
   <si>
-    <t>app.py</t>
-  </si>
-  <si>
-    <t>initial setup</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
     <t>app1,py</t>
   </si>
   <si>
-    <t>solving 'Webhook Delivery failed - 400 Bad request'</t>
-  </si>
-  <si>
     <t>b1</t>
   </si>
   <si>
@@ -63,6 +54,40 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>B7</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>B7 a</t>
+  </si>
+  <si>
+    <t>fixing B7 error - a, b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a. do not alert sell signal
+</t>
+  </si>
+  <si>
+    <t>app0.py</t>
+  </si>
+  <si>
+    <t>app2.py</t>
+  </si>
+  <si>
+    <t>1. XRPUSD becomes XRP</t>
+  </si>
+  <si>
+    <t>initial setup (deleted)</t>
+  </si>
+  <si>
+    <t>fix 'Webhook Delivery failed - 400 Bad request'</t>
+  </si>
+  <si>
+    <t>fix error 1</t>
   </si>
 </sst>
 </file>
@@ -121,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -131,6 +156,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,17 +464,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="53.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.140625" style="5" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="52.28515625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -459,30 +488,50 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2" s="3">
         <v>46116</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="B4" s="3">
         <v>46129</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46130</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -492,7 +541,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
@@ -517,35 +566,60 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B2" s="3">
         <v>46116</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3">
         <v>46129</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46130</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>14</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46130</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix webhook zero qty error and pin dependencies
</commit_message>
<xml_diff>
--- a/app version.xlsx
+++ b/app version.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>Version</t>
   </si>
@@ -50,9 +50,6 @@
     <t>b1a</t>
   </si>
   <si>
-    <t>fixing b1 error</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
@@ -83,11 +80,79 @@
     <t>fix error 1 to change XRPUSD to XRP/USD</t>
   </si>
   <si>
-    <t xml:space="preserve">1. do not alert sell signal
-2. always return qty as </t>
-  </si>
-  <si>
-    <t>fixing B7 error - 1, 2</t>
+    <t>1. do not alert sell signal
+2. always return qty as 1</t>
+  </si>
+  <si>
+    <t>fix b1 error</t>
+  </si>
+  <si>
+    <t>fix B7 error - 1, 2</t>
+  </si>
+  <si>
+    <t>fix B7A error - 1, 2</t>
+  </si>
+  <si>
+    <t>B7 B</t>
+  </si>
+  <si>
+    <t>app3.py</t>
+  </si>
+  <si>
+    <t>2. when selling, possibility of insufficient position
+3. fractional shares wrongly  sent as 0 qty</t>
+  </si>
+  <si>
+    <t>check position to avoild over sell
+fix problem 2</t>
+  </si>
+  <si>
+    <t>B7C</t>
+  </si>
+  <si>
+    <t>To fix the error, sometime Tradinview does not sent alerts when the pinescript triggers buy/sell signal</t>
+  </si>
+  <si>
+    <t>B7D</t>
+  </si>
+  <si>
+    <t>Daily loss kill switch</t>
+  </si>
+  <si>
+    <t>Max trades per day</t>
+  </si>
+  <si>
+    <t>ATR volatility filter</t>
+  </si>
+  <si>
+    <t>Equity-based position sizing</t>
+  </si>
+  <si>
+    <t>Auto risk scaling</t>
+  </si>
+  <si>
+    <t>Just tell me your trading style:</t>
+  </si>
+  <si>
+    <t>Scalp / Intraday / Swing / Crypto ladder?</t>
+  </si>
+  <si>
+    <t>Cater for:Max position cap (prevent overexposure)</t>
+  </si>
+  <si>
+    <t>B7E</t>
+  </si>
+  <si>
+    <t>B8</t>
+  </si>
+  <si>
+    <t>New fifferent full version from ChatGpt replacing B7D</t>
+  </si>
+  <si>
+    <t>Full version from ChatGpt replacing B7D, ChatGpt refers to it as B7c</t>
+  </si>
+  <si>
+    <t>ChatGpt refers to it as B8</t>
   </si>
 </sst>
 </file>
@@ -146,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -159,6 +224,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -464,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
@@ -494,13 +568,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" s="3">
         <v>46116</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>4</v>
@@ -514,24 +588,41 @@
         <v>46129</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3">
         <v>46130</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46131</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -541,88 +632,193 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="53.28515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="53.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="14.140625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="45.85546875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="45.85546875" style="8" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="9">
         <v>46116</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="9">
+        <v>46129</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3">
-        <v>46129</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B6" s="9">
+        <v>46130</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9">
+        <v>46130</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="3">
-        <v>46130</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="3">
-        <v>46130</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>23</v>
+      <c r="E7" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="9">
+        <v>38825</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="9">
+        <v>46131</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="9">
+        <v>46131</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C13" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C14" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C15" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C16" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C18"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C21"/>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="9">
+        <v>46131</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C25" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix alpaca not placing order
</commit_message>
<xml_diff>
--- a/app version.xlsx
+++ b/app version.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="app.py" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
   <si>
     <t>Version</t>
   </si>
@@ -103,56 +103,75 @@
 3. fractional shares wrongly  sent as 0 qty</t>
   </si>
   <si>
+    <t>B7C</t>
+  </si>
+  <si>
+    <t>To fix the error, sometime Tradinview does not sent alerts when the pinescript triggers buy/sell signal</t>
+  </si>
+  <si>
+    <t>B7D</t>
+  </si>
+  <si>
+    <t>Daily loss kill switch</t>
+  </si>
+  <si>
+    <t>Max trades per day</t>
+  </si>
+  <si>
+    <t>ATR volatility filter</t>
+  </si>
+  <si>
+    <t>Equity-based position sizing</t>
+  </si>
+  <si>
+    <t>Auto risk scaling</t>
+  </si>
+  <si>
+    <t>Just tell me your trading style:</t>
+  </si>
+  <si>
+    <t>Scalp / Intraday / Swing / Crypto ladder?</t>
+  </si>
+  <si>
+    <t>Cater for:Max position cap (prevent overexposure)</t>
+  </si>
+  <si>
+    <t>B7E</t>
+  </si>
+  <si>
+    <t>B8</t>
+  </si>
+  <si>
+    <t>New fifferent full version from ChatGpt replacing B7D</t>
+  </si>
+  <si>
+    <t>Full version from ChatGpt replacing B7D, ChatGpt refers to it as B7c</t>
+  </si>
+  <si>
+    <t>ChatGpt refers to it as B8</t>
+  </si>
+  <si>
+    <t>app3a.py</t>
+  </si>
+  <si>
+    <t>this version deoes not check position to avoild over sell
+fix problem 2</t>
+  </si>
+  <si>
     <t>check position to avoild over sell
-fix problem 2</t>
-  </si>
-  <si>
-    <t>B7C</t>
-  </si>
-  <si>
-    <t>To fix the error, sometime Tradinview does not sent alerts when the pinescript triggers buy/sell signal</t>
-  </si>
-  <si>
-    <t>B7D</t>
-  </si>
-  <si>
-    <t>Daily loss kill switch</t>
-  </si>
-  <si>
-    <t>Max trades per day</t>
-  </si>
-  <si>
-    <t>ATR volatility filter</t>
-  </si>
-  <si>
-    <t>Equity-based position sizing</t>
-  </si>
-  <si>
-    <t>Auto risk scaling</t>
-  </si>
-  <si>
-    <t>Just tell me your trading style:</t>
-  </si>
-  <si>
-    <t>Scalp / Intraday / Swing / Crypto ladder?</t>
-  </si>
-  <si>
-    <t>Cater for:Max position cap (prevent overexposure)</t>
-  </si>
-  <si>
-    <t>B7E</t>
-  </si>
-  <si>
-    <t>B8</t>
-  </si>
-  <si>
-    <t>New fifferent full version from ChatGpt replacing B7D</t>
-  </si>
-  <si>
-    <t>Full version from ChatGpt replacing B7D, ChatGpt refers to it as B7c</t>
-  </si>
-  <si>
-    <t>ChatGpt refers to it as B8</t>
+fix problem 2
+fix to ensure fractional shares not wrongly  sent as 0 qty</t>
+  </si>
+  <si>
+    <t>4. Flask app receives the alert
+Flask does not crash
+But Alpaca places no order</t>
+  </si>
+  <si>
+    <t>fix problem 4</t>
+  </si>
+  <si>
+    <t>app4.py</t>
   </si>
 </sst>
 </file>
@@ -538,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" customWidth="1"/>
@@ -614,7 +633,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
@@ -622,7 +641,32 @@
         <v>46131</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>28</v>
+        <v>46</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46132</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46131</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -732,49 +776,49 @@
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="9">
         <v>46131</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="9">
         <v>46131</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C13" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C14" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C15" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C16" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C17" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -782,12 +826,12 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -795,26 +839,26 @@
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="9">
         <v>46131</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C25" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>